<commit_message>
docs: mark finished roadmap items done (M1 pages, M3, M8, M9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -725,7 +725,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Now</t>
+          <t>Done so far</t>
         </is>
       </c>
       <c r="E6" s="6" t="n"/>
@@ -776,7 +776,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Done so far</t>
         </is>
       </c>
       <c r="E7" s="6" t="n"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Now</t>
         </is>
       </c>
       <c r="E8" s="6" t="n"/>
@@ -929,7 +929,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Done so far</t>
         </is>
       </c>
       <c r="E10" s="6" t="n"/>
@@ -980,7 +980,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Later</t>
+          <t>Next</t>
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
@@ -2064,13 +2064,15 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="12" t="n"/>
-      <c r="N13" s="12" t="n"/>
+      <c r="N13" s="12" t="n">
+        <v>46314</v>
+      </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -2125,7 +2127,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -2135,7 +2137,9 @@
       </c>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="12" t="n"/>
-      <c r="N14" s="12" t="n"/>
+      <c r="N14" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -2190,7 +2194,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -2200,7 +2204,9 @@
       </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="12" t="n"/>
-      <c r="N15" s="12" t="n"/>
+      <c r="N15" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -2255,7 +2261,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -2265,7 +2271,9 @@
       </c>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="12" t="n"/>
-      <c r="N16" s="12" t="n"/>
+      <c r="N16" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -2320,13 +2328,15 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="12" t="n"/>
-      <c r="N17" s="12" t="n"/>
+      <c r="N17" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -2381,13 +2391,15 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="12" t="n"/>
-      <c r="N18" s="12" t="n"/>
+      <c r="N18" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -2442,13 +2454,15 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="12" t="n"/>
-      <c r="N19" s="12" t="n"/>
+      <c r="N19" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -3194,13 +3208,15 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
       <c r="M31" s="12" t="n"/>
-      <c r="N31" s="12" t="n"/>
+      <c r="N31" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -3255,7 +3271,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -3265,7 +3281,9 @@
       </c>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="12" t="n"/>
-      <c r="N32" s="12" t="n"/>
+      <c r="N32" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -3320,7 +3338,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
@@ -3330,7 +3348,9 @@
       </c>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="12" t="n"/>
-      <c r="N33" s="12" t="n"/>
+      <c r="N33" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -3385,7 +3405,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -3395,7 +3415,9 @@
       </c>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="12" t="n"/>
-      <c r="N34" s="12" t="n"/>
+      <c r="N34" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -3450,7 +3472,7 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
@@ -3460,13 +3482,19 @@
       </c>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="12" t="n"/>
-      <c r="N35" s="12" t="n"/>
+      <c r="N35" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P35" s="4" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>Accepting invitations in the web app comes with SL-036</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -3641,13 +3669,15 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="12" t="n"/>
-      <c r="N38" s="12" t="n"/>
+      <c r="N38" s="12" t="n">
+        <v>46314</v>
+      </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -3702,7 +3732,7 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -3712,7 +3742,9 @@
       </c>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="12" t="n"/>
-      <c r="N39" s="12" t="n"/>
+      <c r="N39" s="12" t="n">
+        <v>46314</v>
+      </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -5608,7 +5640,7 @@
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K69" s="4" t="inlineStr">
@@ -5618,7 +5650,9 @@
       </c>
       <c r="L69" s="4" t="inlineStr"/>
       <c r="M69" s="12" t="n"/>
-      <c r="N69" s="12" t="n"/>
+      <c r="N69" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O69" s="4" t="inlineStr">
         <is>
           <t>Figma design</t>
@@ -5626,7 +5660,7 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>Dashboard has skeletons; other pages still show a spinner only</t>
+          <t>Every page: grey blocks in its shape while loading; errors as the Figma alert with Try again (or Browse paths)</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5841,7 @@
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
@@ -5817,7 +5851,9 @@
       </c>
       <c r="L72" s="4" t="inlineStr"/>
       <c r="M72" s="12" t="n"/>
-      <c r="N72" s="12" t="n"/>
+      <c r="N72" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O72" s="4" t="inlineStr">
         <is>
           <t>Figma design</t>
@@ -6002,7 +6038,7 @@
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
@@ -6012,7 +6048,9 @@
       </c>
       <c r="L75" s="4" t="inlineStr"/>
       <c r="M75" s="12" t="n"/>
-      <c r="N75" s="12" t="n"/>
+      <c r="N75" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O75" s="4" t="inlineStr">
         <is>
           <t>Figma design</t>
@@ -6067,7 +6105,7 @@
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
@@ -6077,7 +6115,9 @@
       </c>
       <c r="L76" s="4" t="inlineStr"/>
       <c r="M76" s="12" t="n"/>
-      <c r="N76" s="12" t="n"/>
+      <c r="N76" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O76" s="4" t="inlineStr">
         <is>
           <t>Figma design</t>

</xml_diff>

<commit_message>
docs: describe what StudyLog does, list every web page, and finish M1
- README intro says what the app is for; apps/web is no longer "empty for now".
- apps/web/README lists the pages built since: password reset, verify email,
  path preview and settings, analytics, interview ready and settings.
- roadmap.xlsx: SL-019 done (M1 complete); formula results filled in so
  viewers that don't recalculate show the right numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -680,31 +680,31 @@
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="G5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="H5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J5" s="4">
         <f>F5-G5</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K5" s="7">
         <f>IF(F5=0,0,G5/F5)</f>
-        <v/>
-      </c>
-      <c r="L5" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="L5" s="4" t="str">
         <f>IF(F5=0,"Empty",IF(G5=F5,"Done",IF(G5+H5+I5&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="6">
@@ -731,31 +731,31 @@
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="H6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J6" s="4">
         <f>F6-G6</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K6" s="7">
         <f>IF(F6=0,0,G6/F6)</f>
-        <v/>
-      </c>
-      <c r="L6" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="L6" s="4" t="str">
         <f>IF(F6=0,"Empty",IF(G6=F6,"Done",IF(G6+H6+I6&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="7">
@@ -782,31 +782,31 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="G7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="H7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J7" s="4">
         <f>F7-G7</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K7" s="7">
         <f>IF(F7=0,0,G7/F7)</f>
-        <v/>
-      </c>
-      <c r="L7" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="L7" s="4" t="str">
         <f>IF(F7=0,"Empty",IF(G7=F7,"Done",IF(G7+H7+I7&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="8">
@@ -827,37 +827,37 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Now</t>
+          <t>Done so far</t>
         </is>
       </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="H8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J8" s="4">
         <f>F8-G8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K8" s="7">
         <f>IF(F8=0,0,G8/F8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="L8" s="4" t="str">
         <f>IF(F8=0,"Empty",IF(G8=F8,"Done",IF(G8+H8+I8&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="9">
@@ -884,31 +884,31 @@
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="G9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J9" s="4">
         <f>F9-G9</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="K9" s="7">
         <f>IF(F9=0,0,G9/F9)</f>
-        <v/>
-      </c>
-      <c r="L9" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L9" s="4" t="str">
         <f>IF(F9=0,"Empty",IF(G9=F9,"Done",IF(G9+H9+I9&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Not started</v>
       </c>
     </row>
     <row r="10">
@@ -935,31 +935,31 @@
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="G10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="H10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J10" s="4">
         <f>F10-G10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K10" s="7">
         <f>IF(F10=0,0,G10/F10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="L10" s="4" t="str">
         <f>IF(F10=0,"Empty",IF(G10=F10,"Done",IF(G10+H10+I10&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="11">
@@ -980,37 +980,37 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Now</t>
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v/>
-      </c>
-      <c r="L11" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="L11" s="4" t="str">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>In progress</v>
       </c>
     </row>
     <row r="12">
@@ -1037,31 +1037,31 @@
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J12" s="4">
         <f>F12-G12</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K12" s="7">
         <f>IF(F12=0,0,G12/F12)</f>
-        <v/>
-      </c>
-      <c r="L12" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L12" s="4" t="str">
         <f>IF(F12=0,"Empty",IF(G12=F12,"Done",IF(G12+H12+I12&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Not started</v>
       </c>
     </row>
     <row r="13">
@@ -1088,31 +1088,31 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J13" s="4">
         <f>F13-G13</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="K13" s="7">
         <f>IF(F13=0,0,G13/F13)</f>
-        <v/>
-      </c>
-      <c r="L13" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L13" s="4" t="str">
         <f>IF(F13=0,"Empty",IF(G13=F13,"Done",IF(G13+H13+I13&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Not started</v>
       </c>
     </row>
     <row r="14">
@@ -1139,31 +1139,31 @@
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"Done")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"In progress")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J14" s="4">
         <f>F14-G14</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K14" s="7">
         <f>IF(F14=0,0,G14/F14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L14" s="4" t="str">
         <f>IF(F14=0,"Empty",IF(G14=F14,"Done",IF(G14+H14+I14&gt;0,"In progress","Not started")))</f>
-        <v/>
+        <v>Not started</v>
       </c>
     </row>
     <row r="15">
@@ -1178,27 +1178,27 @@
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="8">
         <f>SUM(F5:F14)</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="G15" s="8">
         <f>SUM(G5:G14)</f>
-        <v/>
+        <v>46</v>
       </c>
       <c r="H15" s="8">
         <f>SUM(H5:H14)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I15" s="8">
         <f>SUM(I5:I14)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J15" s="8">
         <f>SUM(J5:J14)</f>
-        <v/>
+        <v>29</v>
       </c>
       <c r="K15" s="10">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v/>
+        <v>0.6133333333333333</v>
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
@@ -1350,9 +1350,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E2,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
@@ -1413,9 +1413,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E3,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1476,9 +1476,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E4,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1539,9 +1539,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E5,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -1602,9 +1602,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E6,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1665,9 +1665,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E7,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -1728,9 +1728,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E8,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -1791,9 +1791,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E9,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
@@ -1854,9 +1854,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E10,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -1917,9 +1917,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E11,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1980,9 +1980,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E12,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Foundations</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -2043,9 +2043,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E13,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -2106,9 +2106,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E14,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -2173,9 +2173,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E15,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
@@ -2240,9 +2240,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E16,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -2307,9 +2307,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E17,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -2370,9 +2370,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E18,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -2433,9 +2433,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E19,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -2496,9 +2496,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E20,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Web: core study loop</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -2517,13 +2517,15 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="12" t="n"/>
-      <c r="N20" s="12" t="n"/>
+      <c r="N20" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -2557,9 +2559,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E21,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -2618,9 +2620,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E22,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
@@ -2683,9 +2685,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E23,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -2744,9 +2746,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E24,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
@@ -2805,9 +2807,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E25,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -2870,9 +2872,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E26,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -2935,9 +2937,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E27,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -3000,9 +3002,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F28" s="4">
+      <c r="F28" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E28,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -3061,9 +3063,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F29" s="4">
+      <c r="F29" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E29,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -3126,9 +3128,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F30" s="4">
+      <c r="F30" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E30,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Production launch</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
@@ -3187,9 +3189,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F31" s="4">
+      <c r="F31" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E31,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Email &amp; accounts</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -3250,9 +3252,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F32" s="4">
+      <c r="F32" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E32,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Email &amp; accounts</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -3317,9 +3319,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F33" s="4">
+      <c r="F33" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E33,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Email &amp; accounts</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -3384,9 +3386,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F34" s="4">
+      <c r="F34" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E34,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Email &amp; accounts</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -3451,9 +3453,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F35" s="4">
+      <c r="F35" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E35,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Email &amp; accounts</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -3522,9 +3524,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F36" s="4">
+      <c r="F36" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E36,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -3583,9 +3585,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F37" s="4">
+      <c r="F37" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E37,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -3648,9 +3650,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F38" s="4">
+      <c r="F38" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E38,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -3711,9 +3713,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F39" s="4">
+      <c r="F39" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E39,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -3778,9 +3780,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F40" s="4">
+      <c r="F40" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E40,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
@@ -3843,9 +3845,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F41" s="4">
+      <c r="F41" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E41,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -3904,9 +3906,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F42" s="4">
+      <c r="F42" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E42,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
@@ -3965,9 +3967,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F43" s="4">
+      <c r="F43" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E43,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Teams &amp; creators (web)</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
@@ -4026,9 +4028,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F44" s="4">
+      <c r="F44" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E44,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Engagement &amp; scale</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -4091,9 +4093,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F45" s="4">
+      <c r="F45" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E45,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Engagement &amp; scale</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -4152,9 +4154,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F46" s="4">
+      <c r="F46" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E46,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Engagement &amp; scale</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -4213,9 +4215,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F47" s="4">
+      <c r="F47" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E47,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Engagement &amp; scale</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
@@ -4274,9 +4276,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F48" s="4">
+      <c r="F48" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E48,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
@@ -4335,9 +4337,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F49" s="4">
+      <c r="F49" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E49,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -4396,9 +4398,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F50" s="4">
+      <c r="F50" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E50,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
@@ -4457,9 +4459,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F51" s="4">
+      <c r="F51" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E51,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -4518,9 +4520,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F52" s="4">
+      <c r="F52" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E52,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4579,9 +4581,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F53" s="4">
+      <c r="F53" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E53,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4640,9 +4642,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F54" s="4">
+      <c r="F54" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E54,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
@@ -4701,9 +4703,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F55" s="4">
+      <c r="F55" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E55,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Quality &amp; docs</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -4762,9 +4764,9 @@
           <t>M7</t>
         </is>
       </c>
-      <c r="F56" s="4">
+      <c r="F56" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E56,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Mobile app</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -4823,9 +4825,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F57" s="4">
+      <c r="F57" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E57,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -4886,9 +4888,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F58" s="4">
+      <c r="F58" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E58,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -4953,9 +4955,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F59" s="4">
+      <c r="F59" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E59,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -5020,9 +5022,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F60" s="4">
+      <c r="F60" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E60,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -5087,9 +5089,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F61" s="4">
+      <c r="F61" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E61,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -5150,9 +5152,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F62" s="4">
+      <c r="F62" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E62,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
@@ -5217,9 +5219,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F63" s="4">
+      <c r="F63" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E63,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -5284,9 +5286,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F64" s="4">
+      <c r="F64" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E64,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
@@ -5351,9 +5353,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F65" s="4">
+      <c r="F65" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E65,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -5418,9 +5420,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F66" s="4">
+      <c r="F66" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E66,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
@@ -5485,9 +5487,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F67" s="4">
+      <c r="F67" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E67,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
@@ -5552,9 +5554,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F68" s="4">
+      <c r="F68" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E68,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
@@ -5619,9 +5621,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F69" s="4">
+      <c r="F69" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E69,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -5690,9 +5692,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F70" s="4">
+      <c r="F70" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E70,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Design system &amp; redesign</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
@@ -5757,9 +5759,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F71" s="4">
+      <c r="F71" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E71,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -5820,9 +5822,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F72" s="4">
+      <c r="F72" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E72,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
@@ -5887,9 +5889,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F73" s="4">
+      <c r="F73" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E73,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -5950,9 +5952,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F74" s="4">
+      <c r="F74" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E74,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
@@ -6017,9 +6019,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F75" s="4">
+      <c r="F75" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E75,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
@@ -6084,9 +6086,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F76" s="4">
+      <c r="F76" s="4" t="str">
         <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E76,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v/>
+        <v>Insights</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: Organizations page, with invitations, members and roles in the web app
- Web: /app/organizations lists invitations for you (accept or decline) and a
  card per organization; /app/organizations/:id has members (search, change
  role, remove, leave), invitations (invite by email, revoke) and published
  paths as tabs, plus rename and delete dialogs (Figma: M4 › Organizations).
- API: GET /organizations adds member and published path counts and the first
  members, for the cards.
- useLoaded moves to api/ and keeps data on screen while reloading the same
  thing.
- e2e: create, invite, accept, change role, rename; last owner can't leave;
  delete needs the name typed. Roadmap: SL-035 and SL-036 done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
@@ -1002,11 +1002,11 @@
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G15" s="8">
         <f>SUM(G5:G14)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H15" s="8">
         <f>SUM(H5:H14)</f>
@@ -1194,11 +1194,11 @@
       </c>
       <c r="J15" s="8">
         <f>SUM(J5:J14)</f>
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K15" s="10">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.6133333333333333</v>
+        <v>0.64</v>
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
@@ -3545,13 +3545,15 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="12" t="n"/>
-      <c r="N36" s="12" t="n"/>
+      <c r="N36" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -3606,7 +3608,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
@@ -3616,7 +3618,9 @@
       </c>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="12" t="n"/>
-      <c r="N37" s="12" t="n"/>
+      <c r="N37" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>

</xml_diff>

<commit_message>
feat(web): report a community path from its preview
- Path preview's About card offers "Report this path" on other people's public
  workspace paths; the dialog takes a reason and optional details (Figma:
  Dialogs › Path preview · report). Reporting twice counts as done.
- e2e: a new user reports Alice's community path; your own path has no link.
  Roadmap: SL-039 done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
@@ -1002,11 +1002,11 @@
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G15" s="8">
         <f>SUM(G5:G14)</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H15" s="8">
         <f>SUM(H5:H14)</f>
@@ -1194,11 +1194,11 @@
       </c>
       <c r="J15" s="8">
         <f>SUM(J5:J14)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K15" s="10">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.64</v>
+        <v>0.6533333333333333</v>
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
@@ -3815,7 +3815,9 @@
       </c>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="12" t="n"/>
-      <c r="N40" s="12" t="n"/>
+      <c r="N40" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>

</xml_diff>

<commit_message>
feat: admin moderation queue, and un-hiding a path hidden by mistake
- Web: /app/admin/reports (superadmins only) lists open reports to dismiss or
  hide the path with a note, and resolved ones with Un-hide (Figma: M4 › Admin ·
  Reports). The "coming soon" page goes: every section is built.
- API: reports include the path's author, whether it's hidden, and who resolved
  them; ?status=resolved lists resolved reports newest first; new
  POST /admin/paths/:pathId/unhide clears publicBlockedAt.
- e2e: hide, un-hide and dismiss as an admin; admin pages are "not found" for
  others. Roadmap: SL-041 and SL-042 done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
@@ -1002,11 +1002,11 @@
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G15" s="8">
         <f>SUM(G5:G14)</f>
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H15" s="8">
         <f>SUM(H5:H14)</f>
@@ -1194,11 +1194,11 @@
       </c>
       <c r="J15" s="8">
         <f>SUM(J5:J14)</f>
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K15" s="10">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.6533333333333333</v>
+        <v>0.68</v>
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
@@ -3933,13 +3933,15 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr"/>
       <c r="M42" s="12" t="n"/>
-      <c r="N42" s="12" t="n"/>
+      <c r="N42" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -3994,13 +3996,15 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr"/>
       <c r="M43" s="12" t="n"/>
-      <c r="N43" s="12" t="n"/>
+      <c r="N43" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>

</xml_diff>

<commit_message>
feat: admin global catalog editor in the web app
- Web: /app/admin/catalog (superadmins only) lists official paths and items
  (?tab=items) with status, size and last update; new path and item dialogs;
  publish, move to draft, archive and delete from each row's menu (Figma:
  M4 › Admin · Catalog, States › Admin · Items). Paths open in the path builder,
  in global catalog mode. Admin now opens on the catalog, with Reports beside it.
- Item form fields move to ItemFields so My paths and the admin catalog share
  them; StatusBadge and catalog status labels are shared too.
- API: GET /admin/catalog/paths adds moduleCount and itemCount; GET
  /admin/catalog/items adds topicCount (ManagedLearningPath, ManagedItem).
- e2e: a superadmin builds a draft path and item, publishes parts and deletes
  them. Roadmap: SL-040 done, M4 complete.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -980,7 +980,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Now</t>
+          <t>Done so far</t>
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
@@ -990,7 +990,7 @@
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
@@ -1002,15 +1002,15 @@
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v>0.875</v>
+        <v>1.0</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
-        <v>In progress</v>
+        <v>Done</v>
       </c>
     </row>
     <row r="12">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G15" s="8">
         <f>SUM(G5:G14)</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H15" s="8">
         <f>SUM(H5:H14)</f>
@@ -1194,11 +1194,11 @@
       </c>
       <c r="J15" s="8">
         <f>SUM(J5:J14)</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K15" s="10">
         <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.68</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="L15" s="9" t="n"/>
     </row>
@@ -3872,13 +3872,15 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr"/>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="12" t="n"/>
-      <c r="N41" s="12" t="n"/>
+      <c r="N41" s="12" t="n">
+        <v>46318</v>
+      </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>

</xml_diff>

<commit_message>
chore: update the roadmap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P76" headerRowCount="1">
-  <autoFilter ref="A1:P76"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P105" headerRowCount="1">
+  <autoFilter ref="A1:P105"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Title"/>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -680,31 +680,31 @@
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>11</v>
+        <v/>
       </c>
       <c r="G5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"Done")</f>
-        <v>11</v>
+        <v/>
       </c>
       <c r="H5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I5" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A5,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J5" s="4">
         <f>F5-G5</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K5" s="7">
         <f>IF(F5=0,0,G5/F5)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4">
         <f>IF(F5=0,"Empty",IF(G5=F5,"Done",IF(G5+H5+I5&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -731,31 +731,31 @@
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>14</v>
+        <v/>
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"Done")</f>
-        <v>14</v>
+        <v/>
       </c>
       <c r="H6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I6" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A6,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J6" s="4">
         <f>F6-G6</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K6" s="7">
         <f>IF(F6=0,0,G6/F6)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L6" s="4">
         <f>IF(F6=0,"Empty",IF(G6=F6,"Done",IF(G6+H6+I6&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -782,31 +782,31 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>6</v>
+        <v/>
       </c>
       <c r="G7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"Done")</f>
-        <v>6</v>
+        <v/>
       </c>
       <c r="H7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I7" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A7,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J7" s="4">
         <f>F7-G7</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K7" s="7">
         <f>IF(F7=0,0,G7/F7)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4">
         <f>IF(F7=0,"Empty",IF(G7=F7,"Done",IF(G7+H7+I7&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -833,31 +833,31 @@
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="G8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"Done")</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="H8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I8" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A8,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J8" s="4">
         <f>F8-G8</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K8" s="7">
         <f>IF(F8=0,0,G8/F8)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4">
         <f>IF(F8=0,"Empty",IF(G8=F8,"Done",IF(G8+H8+I8&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -884,31 +884,31 @@
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>10</v>
+        <v/>
       </c>
       <c r="G9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"Done")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="H9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I9" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A9,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J9" s="4">
         <f>F9-G9</f>
-        <v>10</v>
+        <v/>
       </c>
       <c r="K9" s="7">
         <f>IF(F9=0,0,G9/F9)</f>
-        <v>0.0</v>
-      </c>
-      <c r="L9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="4">
         <f>IF(F9=0,"Empty",IF(G9=F9,"Done",IF(G9+H9+I9&gt;0,"In progress","Not started")))</f>
-        <v>Not started</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -935,31 +935,31 @@
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="G10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"Done")</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="H10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I10" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A10,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J10" s="4">
         <f>F10-G10</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K10" s="7">
         <f>IF(F10=0,0,G10/F10)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="4">
         <f>IF(F10=0,"Empty",IF(G10=F10,"Done",IF(G10+H10+I10&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -986,31 +986,31 @@
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="G11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Done")</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="H11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I11" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A11,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J11" s="4">
         <f>F11-G11</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K11" s="7">
         <f>IF(F11=0,0,G11/F11)</f>
-        <v>1.0</v>
-      </c>
-      <c r="L11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="4">
         <f>IF(F11=0,"Empty",IF(G11=F11,"Done",IF(G11+H11+I11&gt;0,"In progress","Not started")))</f>
-        <v>Done</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1037,31 +1037,31 @@
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="G12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"Done")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="H12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I12" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A12,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J12" s="4">
         <f>F12-G12</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="K12" s="7">
         <f>IF(F12=0,0,G12/F12)</f>
-        <v>0.0</v>
-      </c>
-      <c r="L12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L12" s="4">
         <f>IF(F12=0,"Empty",IF(G12=F12,"Done",IF(G12+H12+I12&gt;0,"In progress","Not started")))</f>
-        <v>Not started</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1088,31 +1088,31 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="G13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"Done")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="H13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A13,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J13" s="4">
         <f>F13-G13</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="K13" s="7">
         <f>IF(F13=0,0,G13/F13)</f>
-        <v>0.0</v>
-      </c>
-      <c r="L13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L13" s="4">
         <f>IF(F13=0,"Empty",IF(G13=F13,"Done",IF(G13+H13+I13&gt;0,"In progress","Not started")))</f>
-        <v>Not started</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1139,71 +1139,173 @@
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="G14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"Done")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="H14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"In progress")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(Backlog!$E$2:$E$500,$A14,Backlog!$J$2:$J$500,"Blocked")</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J14" s="4">
         <f>F14-G14</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="K14" s="7">
         <f>IF(F14=0,0,G14/F14)</f>
-        <v>0.0</v>
-      </c>
-      <c r="L14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L14" s="4">
         <f>IF(F14=0,"Empty",IF(G14=F14,"Done",IF(G14+H14+I14&gt;0,"In progress","Not started")))</f>
-        <v>Not started</v>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Platform admin</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Superadmin tools to run the platform: users, an overview, organizations and an audit log</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A15,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A15,Backlog!$J$2:$J$500,"Done")</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A15,Backlog!$J$2:$J$500,"In progress")</f>
+        <v/>
+      </c>
+      <c r="I15" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A15,Backlog!$J$2:$J$500,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="J15" s="4">
+        <f>F15-G15</f>
+        <v/>
+      </c>
+      <c r="K15" s="7">
+        <f>IF(F15=0,0,G15/F15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="4">
+        <f>IF(F15=0,"Empty",IF(G15=F15,"Done",IF(G15+H15+I15&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Launch &amp; growth</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>The first users: official paths to study, outreach, feedback and the numbers that show what works</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A16,Backlog!$J$2:$J$500,"&lt;&gt;Won't do")</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A16,Backlog!$J$2:$J$500,"Done")</f>
+        <v/>
+      </c>
+      <c r="H16" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A16,Backlog!$J$2:$J$500,"In progress")</f>
+        <v/>
+      </c>
+      <c r="I16" s="4">
+        <f>COUNTIFS(Backlog!$E$2:$E$500,$A16,Backlog!$J$2:$J$500,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="J16" s="4">
+        <f>F16-G16</f>
+        <v/>
+      </c>
+      <c r="K16" s="7">
+        <f>IF(F16=0,0,G16/F16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="4">
+        <f>IF(F16=0,"Empty",IF(G16=F16,"Done",IF(G16+H16+I16&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="8">
-        <f>SUM(F5:F14)</f>
-        <v>75</v>
-      </c>
-      <c r="G15" s="8">
-        <f>SUM(G5:G14)</f>
-        <v>52</v>
-      </c>
-      <c r="H15" s="8">
-        <f>SUM(H5:H14)</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="8">
-        <f>SUM(I5:I14)</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="8">
-        <f>SUM(J5:J14)</f>
-        <v>23</v>
-      </c>
-      <c r="K15" s="10">
-        <f>IF(F15=0,0,G15/F15)</f>
-        <v>0.6933333333333334</v>
-      </c>
-      <c r="L15" s="9" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="8">
+        <f>SUM(F5:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="8">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="8">
+        <f>SUM(H5:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="8">
+        <f>SUM(I5:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="8">
+        <f>SUM(J5:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="10">
+        <f>IF(F17=0,0,G17/F17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="9" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L5:L14">
+  <conditionalFormatting sqref="L5:L16">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L5="Done"</formula>
     </cfRule>
@@ -1221,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1350,9 +1452,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F2" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E2,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F2" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E2,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
@@ -1413,9 +1515,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F3" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E3,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F3" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E3,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1476,9 +1578,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F4" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E4,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F4" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E4,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1539,9 +1641,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F5" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E5,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F5" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E5,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -1602,9 +1704,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F6" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E6,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F6" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E6,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1665,9 +1767,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F7" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E7,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F7" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E7,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -1728,9 +1830,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F8" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E8,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F8" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E8,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -1791,9 +1893,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F9" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E9,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F9" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E9,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
@@ -1854,9 +1956,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F10" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E10,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F10" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E10,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -1917,9 +2019,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F11" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E11,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F11" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E11,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
@@ -1980,9 +2082,9 @@
           <t>M0</t>
         </is>
       </c>
-      <c r="F12" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E12,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Foundations</v>
+      <c r="F12" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E12,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -2043,9 +2145,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F13" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E13,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F13" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E13,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -2106,9 +2208,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F14" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E14,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F14" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E14,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -2173,9 +2275,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F15" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E15,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F15" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E15,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
@@ -2240,9 +2342,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F16" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E16,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F16" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E16,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -2307,9 +2409,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F17" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E17,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F17" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E17,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
@@ -2370,9 +2472,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F18" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E18,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F18" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E18,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
@@ -2433,9 +2535,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F19" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E19,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F19" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E19,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -2496,9 +2598,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="F20" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E20,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Web: core study loop</v>
+      <c r="F20" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E20,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -2559,9 +2661,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F21" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E21,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F21" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E21,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -2580,19 +2682,25 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="12" t="n"/>
-      <c r="N21" s="12" t="n"/>
+      <c r="N21" s="12" t="n">
+        <v>46319</v>
+      </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>PRs only: lint, build, unit tests with coverage (posted on the PR) and the Playwright UI tests; turbo and Playwright caching. migration:generate --check and mutation testing moved to SL-080.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2620,9 +2728,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F22" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E22,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F22" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E22,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
@@ -2641,7 +2749,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -2657,7 +2765,11 @@
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>Ruleset ready to import (master-ruleset.json: PRs only, both CI checks, branch up to date, no force pushes). Done once it shows Active under Settings → Rules.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2685,9 +2797,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F23" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E23,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F23" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E23,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -2746,9 +2858,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F24" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E24,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F24" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E24,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
@@ -2767,19 +2879,25 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="12" t="n"/>
-      <c r="N24" s="12" t="n"/>
+      <c r="N24" s="12" t="n">
+        <v>46319</v>
+      </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Images built by GitHub Actions to GHCR; deployed on Civo k3s (deploy/civo), live at https://gradiaqo.com. Migrations run in an init container before the API starts.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2807,9 +2925,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F25" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E25,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F25" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E25,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -2828,7 +2946,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -2838,13 +2956,19 @@
       </c>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="12" t="n"/>
-      <c r="N25" s="12" t="n"/>
+      <c r="N25" s="12" t="n">
+        <v>46319</v>
+      </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>deploy/k8s/config.env: production, secure cookies, Swagger off, TRUST_PROXY=2 (Traefik + Caddy). SMTP on port 2525: Civo blocks 25/465/587.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2872,9 +2996,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F26" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E26,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F26" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E26,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -2937,9 +3061,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F27" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E27,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F27" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E27,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -3002,9 +3126,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F28" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E28,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F28" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E28,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -3063,9 +3187,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F29" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E29,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F29" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E29,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -3128,9 +3252,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="F30" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E30,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Production launch</v>
+      <c r="F30" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E30,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
@@ -3189,9 +3313,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F31" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E31,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Email &amp; accounts</v>
+      <c r="F31" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E31,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -3252,9 +3376,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F32" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E32,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Email &amp; accounts</v>
+      <c r="F32" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E32,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -3319,9 +3443,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F33" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E33,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Email &amp; accounts</v>
+      <c r="F33" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E33,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
@@ -3386,9 +3510,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F34" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E34,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Email &amp; accounts</v>
+      <c r="F34" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E34,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -3453,9 +3577,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="F35" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E35,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Email &amp; accounts</v>
+      <c r="F35" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E35,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -3524,9 +3648,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F36" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E36,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F36" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E36,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -3587,9 +3711,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F37" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E37,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F37" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E37,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -3654,9 +3778,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F38" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E38,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F38" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E38,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -3717,9 +3841,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F39" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E39,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F39" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E39,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
@@ -3784,9 +3908,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F40" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E40,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F40" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E40,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
@@ -3851,9 +3975,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F41" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E41,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F41" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E41,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -3914,9 +4038,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F42" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E42,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F42" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E42,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
@@ -3977,9 +4101,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="F43" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E43,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Teams &amp; creators (web)</v>
+      <c r="F43" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E43,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
@@ -4040,9 +4164,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F44" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E44,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Engagement &amp; scale</v>
+      <c r="F44" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E44,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
@@ -4105,9 +4229,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F45" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E45,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Engagement &amp; scale</v>
+      <c r="F45" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E45,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
@@ -4166,9 +4290,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F46" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E46,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Engagement &amp; scale</v>
+      <c r="F46" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E46,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
@@ -4227,9 +4351,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="F47" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E47,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Engagement &amp; scale</v>
+      <c r="F47" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E47,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
@@ -4288,9 +4412,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F48" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E48,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F48" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E48,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
@@ -4349,9 +4473,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F49" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E49,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F49" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E49,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
@@ -4410,9 +4534,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F50" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E50,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F50" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E50,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
@@ -4471,9 +4595,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F51" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E51,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F51" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E51,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -4532,9 +4656,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F52" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E52,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F52" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E52,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -4593,9 +4717,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F53" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E53,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F53" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E53,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
@@ -4654,9 +4778,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F54" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E54,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F54" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E54,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
@@ -4715,9 +4839,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="F55" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E55,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Quality &amp; docs</v>
+      <c r="F55" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E55,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -4776,9 +4900,9 @@
           <t>M7</t>
         </is>
       </c>
-      <c r="F56" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E56,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Mobile app</v>
+      <c r="F56" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E56,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -4837,9 +4961,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F57" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E57,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F57" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E57,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -4900,9 +5024,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F58" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E58,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F58" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E58,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -4967,9 +5091,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F59" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E59,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F59" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E59,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -5034,9 +5158,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F60" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E60,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F60" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E60,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
@@ -5101,9 +5225,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F61" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E61,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F61" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E61,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -5164,9 +5288,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F62" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E62,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F62" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E62,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
@@ -5231,9 +5355,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F63" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E63,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F63" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E63,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -5298,9 +5422,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F64" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E64,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F64" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E64,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
@@ -5365,9 +5489,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F65" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E65,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F65" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E65,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
@@ -5432,9 +5556,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F66" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E66,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F66" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E66,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
@@ -5499,9 +5623,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F67" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E67,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F67" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E67,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
@@ -5566,9 +5690,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F68" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E68,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F68" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E68,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
@@ -5633,9 +5757,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F69" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E69,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F69" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E69,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
@@ -5704,9 +5828,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="F70" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E70,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Design system &amp; redesign</v>
+      <c r="F70" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E70,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
@@ -5771,9 +5895,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F71" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E71,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F71" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E71,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -5834,9 +5958,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F72" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E72,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F72" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E72,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
@@ -5901,9 +6025,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F73" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E73,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F73" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E73,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -5964,9 +6088,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F74" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E74,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F74" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E74,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
@@ -6031,9 +6155,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F75" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E75,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F75" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E75,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
@@ -6098,9 +6222,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="F76" s="4" t="str">
-        <f>IFERROR(INDEX(Roadmap!$B$5:$B$14,MATCH(E76,Roadmap!$A$5:$A$14,0)),"")</f>
-        <v>Insights</v>
+      <c r="F76" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E76,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
@@ -6142,6 +6266,1887 @@
           <t>API unit tests done (100%); UI tests come with the pages</t>
         </is>
       </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>SL-076</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Database backups off the server</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Nightly pg_dump as a Kubernetes CronJob, uploaded to object storage outside Civo (Cloudflare R2 or Backblaze B2 free tier, or Civo Object Store about $5.43/month); keep 30 days; test a restore</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F77" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E77,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>SL-023</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="n"/>
+      <c r="M77" s="12" t="n"/>
+      <c r="N77" s="12" t="n"/>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>The database volume is set to Retain, but that is not a backup. Decide the storage first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>SL-077</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Finish Brevo email authentication</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Merge SPF into one record (v=spf1 include:zoho.in include:spf.brevo.com ~all); Authenticate the domain in Brevo; check DKIM and DMARC pass in Gmail ("Show original")</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F78" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E78,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="n"/>
+      <c r="L78" s="4" t="n"/>
+      <c r="M78" s="12" t="n"/>
+      <c r="N78" s="12" t="n"/>
+      <c r="O78" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P78" s="4" t="inlineStr">
+        <is>
+          <t>brevo-code, DKIM (brevo1/brevo2) and DMARC records are live; SPF still only has Zoho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>SL-078</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Redirect www to gradiaqo.com</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>www.gradiaqo.com has a CNAME but no certificate or route: add it to the Ingress and certificate, redirecting to the bare domain</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F79" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E79,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>SL-023</t>
+        </is>
+      </c>
+      <c r="L79" s="4" t="n"/>
+      <c r="M79" s="12" t="n"/>
+      <c r="N79" s="12" t="n"/>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>SL-079</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Uptime monitoring</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>External check on https://gradiaqo.com/health (e.g. UptimeRobot or Better Stack) with email alerts</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F80" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E80,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>SL-023</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="n"/>
+      <c r="M80" s="12" t="n"/>
+      <c r="N80" s="12" t="n"/>
+      <c r="O80" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>SL-080</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>CI: migration check and mutation testing</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>The parts of SL-020 not built yet: migration:generate --check (entities and migrations agree) and incremental mutation testing on pull requests</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F81" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E81,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr">
+        <is>
+          <t>SL-020</t>
+        </is>
+      </c>
+      <c r="L81" s="4" t="n"/>
+      <c r="M81" s="12" t="n"/>
+      <c r="N81" s="12" t="n"/>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>SL-081</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Shorter SMTP timeouts</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>When the mail server can't be reached, signup waits about 30 s for the connection to time out; set nodemailer connection and greeting timeouts of a few seconds</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F82" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E82,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="n"/>
+      <c r="L82" s="4" t="n"/>
+      <c r="M82" s="12" t="n"/>
+      <c r="N82" s="12" t="n"/>
+      <c r="O82" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P82" s="4" t="inlineStr">
+        <is>
+          <t>Seen on the first production signup, before SMTP moved to port 2525.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>SL-082</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Rebrand the app to Gradiaqo</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>The web app, page titles, homepage and image names still say StudyLog; emails already say Gradiaqo (BRAND in apps/api/src/mail/templates.ts)</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F83" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E83,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="n"/>
+      <c r="L83" s="4" t="n"/>
+      <c r="M83" s="12" t="n"/>
+      <c r="N83" s="12" t="n"/>
+      <c r="O83" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>SL-083</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>CLI: user:promote</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>yarn cli user:promote &lt;email&gt; (and --demote) to make a superadmin without SQL; documented in deploy/k8s/README.md</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F84" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E84,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="n"/>
+      <c r="L84" s="4" t="n"/>
+      <c r="M84" s="12" t="n"/>
+      <c r="N84" s="12" t="n"/>
+      <c r="O84" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P84" s="4" t="inlineStr">
+        <is>
+          <t>The first superadmin was set with a manual UPDATE on 2026-10-24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>SL-084</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Admin users API</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/users (search by email or name, paginated; verified, role, created, last login if tracked), PATCH platform role, DELETE an account (spam)</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F85" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E85,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="n"/>
+      <c r="L85" s="4" t="n"/>
+      <c r="M85" s="12" t="n"/>
+      <c r="N85" s="12" t="n"/>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>SL-085</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Admin users page</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>/app/admin/users: search, verified badge, promote or demote superadmin, remove an account with confirmation; sidebar link</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F86" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E86,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr">
+        <is>
+          <t>SL-084</t>
+        </is>
+      </c>
+      <c r="L86" s="4" t="n"/>
+      <c r="M86" s="12" t="n"/>
+      <c r="N86" s="12" t="n"/>
+      <c r="O86" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>SL-086</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Admin platform overview</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Sign-ups per day, active learners, verified vs unverified accounts, most-enrolled paths; API and page; becomes the /app/admin landing page (today it redirects to the catalog)</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F87" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E87,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="n"/>
+      <c r="L87" s="4" t="n"/>
+      <c r="M87" s="12" t="n"/>
+      <c r="N87" s="12" t="n"/>
+      <c r="O87" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>SL-087</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Admin organizations oversight</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>List every organization with its members and paths, for abuse and support requests; API and page</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F88" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E88,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="n"/>
+      <c r="L88" s="4" t="n"/>
+      <c r="M88" s="12" t="n"/>
+      <c r="N88" s="12" t="n"/>
+      <c r="O88" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>SL-088</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Admin audit log</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Record who hid, un-hid, published, archived or promoted what and when; a page to browse it</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F89" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E89,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="n"/>
+      <c r="L89" s="4" t="n"/>
+      <c r="M89" s="12" t="n"/>
+      <c r="N89" s="12" t="n"/>
+      <c r="O89" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>SL-089</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>SEO basics</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>A title and description per public page (home, login, signup) under the Gradiaqo name; Open Graph and Twitter tags with a 1200×630 share image, so shared links show a card; robots.txt (allow /, disallow /app/) and sitemap.xml served by Caddy; noindex on /app pages; favicon.ico</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F90" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E90,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr">
+        <is>
+          <t>SL-082</t>
+        </is>
+      </c>
+      <c r="L90" s="4" t="n"/>
+      <c r="M90" s="12" t="n"/>
+      <c r="N90" s="12" t="n"/>
+      <c r="O90" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P90" s="4" t="inlineStr">
+        <is>
+          <t>Today every page is titled "StudyLog", there are no preview tags, and robots.txt and sitemap.xml return the API's 404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>SL-090</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Pre-render the homepage</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Render the homepage to static HTML at build time, so search engines and link previews (WhatsApp, LinkedIn, Slack) see its content instead of an empty &lt;div id="root"&gt;</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F91" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E91,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr">
+        <is>
+          <t>SL-089</t>
+        </is>
+      </c>
+      <c r="L91" s="4" t="n"/>
+      <c r="M91" s="12" t="n"/>
+      <c r="N91" s="12" t="n"/>
+      <c r="O91" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>SL-091</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Google Search Console</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Verify gradiaqo.com with a DNS TXT record at Hostinger, submit sitemap.xml, check indexing and search queries</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F92" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E92,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr">
+        <is>
+          <t>SL-089</t>
+        </is>
+      </c>
+      <c r="L92" s="4" t="n"/>
+      <c r="M92" s="12" t="n"/>
+      <c r="N92" s="12" t="n"/>
+      <c r="O92" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>SL-092</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Public learning-path pages</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Read-only public pages for selected official paths (e.g. DSA, system design) with "Sign up to start": the pages people would find through search. Today the catalog is behind login</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="F93" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E93,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr">
+        <is>
+          <t>SL-089</t>
+        </is>
+      </c>
+      <c r="L93" s="4" t="n"/>
+      <c r="M93" s="12" t="n"/>
+      <c r="N93" s="12" t="n"/>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P93" s="4" t="inlineStr">
+        <is>
+          <t>A product decision first: which paths, and how much of each to show logged out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>SL-093</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Dark theme design in Figma</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Dark mode for the Figma variables and a pass over the screens (charts, badges, dialogs), so the dark values are designed rather than guessed</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="F94" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E94,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr">
+        <is>
+          <t>SL-056</t>
+        </is>
+      </c>
+      <c r="L94" s="4" t="n"/>
+      <c r="M94" s="12" t="n"/>
+      <c r="N94" s="12" t="n"/>
+      <c r="O94" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>SL-094</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Dark theme in the web app</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Follow the system setting by default, with Light / Dark / System in Settings (remembered); set before the first paint so pages don't flash; check every page, chart and dialog in both themes; UI tests for the switch</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="F95" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E95,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>SL-093</t>
+        </is>
+      </c>
+      <c r="L95" s="4" t="n"/>
+      <c r="M95" s="12" t="n"/>
+      <c r="N95" s="12" t="n"/>
+      <c r="O95" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P95" s="4" t="inlineStr">
+        <is>
+          <t>The dark tokens already exist in apps/web/src/index.css (:root[data-theme='dark']) but nothing switches them on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Publish the first official paths</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>3–5 interview-prep paths in the admin catalog editor, well ordered with good free resources: DSA (arrays to DP), system design basics, SQL, JavaScript/React or CS fundamentals (OS, DBMS, networks). Quality over quantity</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F96" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E96,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="n"/>
+      <c r="L96" s="4" t="n"/>
+      <c r="M96" s="12" t="n"/>
+      <c r="N96" s="12" t="n"/>
+      <c r="O96" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P96" s="4" t="inlineStr">
+        <is>
+          <t>On 2026-10-24 production had 0 learning paths: a new user finds nothing to study. Do this before any outreach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>SL-096</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Feedback link and early-user group</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>A "Feedback" link in the app (to a form) and a WhatsApp or Telegram group for early users</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F97" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E97,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="n"/>
+      <c r="L97" s="4" t="n"/>
+      <c r="M97" s="12" t="n"/>
+      <c r="N97" s="12" t="n"/>
+      <c r="O97" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>SL-097</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>First 10–30 users, one by one</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Personal messages to friends, juniors and ex-colleagues preparing for interviews ("try the DSA path for a week and tell me what's annoying"); watch 3–5 of them sign up and enrol over a call</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F98" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E98,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L98" s="4" t="n"/>
+      <c r="M98" s="12" t="n"/>
+      <c r="N98" s="12" t="n"/>
+      <c r="O98" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P98" s="4" t="inlineStr">
+        <is>
+          <t>Before: SL-082 rebrand, SL-089 link previews, SL-077 SPF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>SL-098</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Sign-up source tracking</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Keep ?ref= (linkedin, reddit, a college group…) through signup and store it on the account; shown in the admin overview</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F99" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E99,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>SL-086</t>
+        </is>
+      </c>
+      <c r="L99" s="4" t="n"/>
+      <c r="M99" s="12" t="n"/>
+      <c r="N99" s="12" t="n"/>
+      <c r="O99" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>SL-099</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Weekly growth numbers</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>Every week: sign-ups, activation (verified and enrolled in a path) and week-2 retention (studied again in the second week); fix retention before pushing more traffic</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F100" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E100,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>SL-086</t>
+        </is>
+      </c>
+      <c r="L100" s="4" t="n"/>
+      <c r="M100" s="12" t="n"/>
+      <c r="N100" s="12" t="n"/>
+      <c r="O100" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>SL-100</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Build in public on LinkedIn</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>A weekly post about building Gradiaqo: features, the stack, the $12/month Civo setup, lessons learned</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F101" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E101,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="n"/>
+      <c r="L101" s="4" t="n"/>
+      <c r="M101" s="12" t="n"/>
+      <c r="N101" s="12" t="n"/>
+      <c r="O101" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P101" s="4" t="inlineStr">
+        <is>
+          <t>Ongoing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>SL-101</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>Posts in developer communities</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>Useful posts first (e.g. "the DSA order I'd follow for 8 weeks") with the app at the end: r/developersIndia, r/leetcode, college placement-prep WhatsApp/Telegram/Discord groups. Check each community's self-promotion rules</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F102" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E102,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L102" s="4" t="n"/>
+      <c r="M102" s="12" t="n"/>
+      <c r="N102" s="12" t="n"/>
+      <c r="O102" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>SL-102</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Study groups and coding clubs</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Offer clubs and study groups an organization: shared paths and each other's progress. One club admin can bring 30 users</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F103" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E103,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L103" s="4" t="n"/>
+      <c r="M103" s="12" t="n"/>
+      <c r="N103" s="12" t="n"/>
+      <c r="O103" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P103" s="4" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>SL-103</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Product Hunt and Peerlist launch</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Launch once there are about 50 active users and a few testimonials</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F104" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E104,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="inlineStr">
+        <is>
+          <t>SL-097</t>
+        </is>
+      </c>
+      <c r="L104" s="4" t="n"/>
+      <c r="M104" s="12" t="n"/>
+      <c r="N104" s="12" t="n"/>
+      <c r="O104" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>SL-104</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Invite a study buddy</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>Referral: invite a friend to study the same path together; once week-2 retention is good</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F105" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E105,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>SL-099</t>
+        </is>
+      </c>
+      <c r="L105" s="4" t="n"/>
+      <c r="M105" s="12" t="n"/>
+      <c r="N105" s="12" t="n"/>
+      <c r="O105" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P105" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P500">
@@ -6172,10 +8177,10 @@
       <formula1>=Lists!$D$2:$D$4</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$E$2:$E$10</formula1>
+      <formula1>=Lists!$E$2:$E$12</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Roadmap!$A$5:$A$14</formula1>
+      <formula1>=Roadmap!$A$5:$A$16</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6240,7 +8245,7 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Type in the first empty row under the table: it grows automatically. Use the next ID (SL-0xx) and pick a Milestone (M0–M9).</t>
+          <t>Type in the first empty row under the table: it grows automatically. Use the next ID (SL-0xx) and pick a Milestone (M0–M11).</t>
         </is>
       </c>
     </row>
@@ -6354,7 +8359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6527,6 +8532,20 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(roadmap): SL-105 AI Engineer path; SL-021, 077, 093, 094 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P105" headerRowCount="1">
-  <autoFilter ref="A1:P105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P106" headerRowCount="1">
+  <autoFilter ref="A1:P106"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Title"/>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:P106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -2759,7 +2759,9 @@
       </c>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="12" t="n"/>
-      <c r="N22" s="12" t="n"/>
+      <c r="N22" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
           <t>README roadmap</t>
@@ -2767,7 +2769,7 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Ruleset ready to import (master-ruleset.json: PRs only, both CI checks, branch up to date, no force pushes). Done once it shows Active under Settings → Rules.</t>
+          <t>Ruleset (branchruleset.json) active on master, checked through the GitHub API on 2026-10-26: no deletion, no force pushes, PRs only, both CI checks required.</t>
         </is>
       </c>
     </row>
@@ -6383,13 +6385,15 @@
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K78" s="4" t="n"/>
       <c r="L78" s="4" t="n"/>
       <c r="M78" s="12" t="n"/>
-      <c r="N78" s="12" t="n"/>
+      <c r="N78" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O78" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6397,7 +6401,7 @@
       </c>
       <c r="P78" s="4" t="inlineStr">
         <is>
-          <t>brevo-code, DKIM (brevo1/brevo2) and DMARC records are live; SPF still only has Zoho.</t>
+          <t>Checked in public DNS on 2026-10-26: one SPF record with Zoho and Brevo, DKIM brevo1/brevo2, DMARC and brevo-code all live. Later: DMARC p=none → p=quarantine after a few weeks of clean reports.</t>
         </is>
       </c>
     </row>
@@ -7411,7 +7415,7 @@
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
@@ -7421,13 +7425,19 @@
       </c>
       <c r="L94" s="4" t="n"/>
       <c r="M94" s="12" t="n"/>
-      <c r="N94" s="12" t="n"/>
+      <c r="N94" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O94" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="P94" s="4" t="n"/>
+      <c r="P94" s="4" t="inlineStr">
+        <is>
+          <t>Figma Starter plan allows one mode per collection, so dark is a separate "Color – Dark" collection (same names and CSS names; edit both together), plus Shadow/Dark/* styles and color/bg/scrim. 11 dark screens in Screens – Web › Dark · key screens.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -7476,7 +7486,7 @@
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
@@ -7486,7 +7496,9 @@
       </c>
       <c r="L95" s="4" t="n"/>
       <c r="M95" s="12" t="n"/>
-      <c r="N95" s="12" t="n"/>
+      <c r="N95" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O95" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7494,7 +7506,7 @@
       </c>
       <c r="P95" s="4" t="inlineStr">
         <is>
-          <t>The dark tokens already exist in apps/web/src/index.css (:root[data-theme='dark']) but nothing switches them on.</t>
+          <t>Settings › Appearance (Light / Dark / System), remembered per browser; src/theme/theme.ts and a pre-paint script in index.html. Dark fixes: accent hover violet/600 (AA), --color-scrim, accent-tint CTA band. Deployed to gradiaqo.com 2026-10-26.</t>
         </is>
       </c>
     </row>
@@ -8147,6 +8159,75 @@
         </is>
       </c>
       <c r="P105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>SL-105</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer learning path</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>An official path for building products on LLMs: how models work, model APIs, prompting, embeddings, RAG, tools and agents (MCP), evals, open models and fine-tuning, production and security, and a capstone. Free resources plus a project in most modules</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F106" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E106,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K106" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L106" s="4" t="n"/>
+      <c r="M106" s="12" t="n"/>
+      <c r="N106" s="12" t="n"/>
+      <c r="O106" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P106" s="4" t="inlineStr">
+        <is>
+          <t>content/paths/ai-engineer.yaml: 10 modules, 23 topics, 65 items (15 optional, 12 exercises), about 2–3 months at an hour a day. Passes the importer's parser; all non-YouTube links returned 200 on 2026-10-28, the 5 YouTube links still to check by hand. Next: import on production, check in Admin › Catalog, publish.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P500">

</xml_diff>

<commit_message>
chore(roadmap): SL-106 System Design path
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P106" headerRowCount="1">
-  <autoFilter ref="A1:P106"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P107" headerRowCount="1">
+  <autoFilter ref="A1:P107"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Title"/>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8226,6 +8226,75 @@
       <c r="P106" s="4" t="inlineStr">
         <is>
           <t>content/paths/ai-engineer.yaml: 10 modules, 23 topics, 65 items (15 optional, 12 exercises), about 2–3 months at an hour a day. Passes the importer's parser; all non-YouTube links returned 200 on 2026-10-28, the 5 YouTube links still to check by hand. Next: import on production, check in Admin › Catalog, publish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>SL-106</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>System Design learning path</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>An official path for system design interviews: the 45-minute framework and estimation, networking and APIs, databases (indexes, replication, sharding), caching and CDNs, queues and streams, distributed-systems trade-offs, reliability, 12 classic designs with answer notes, and mock interviews</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F107" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E107,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L107" s="4" t="n"/>
+      <c r="M107" s="12" t="n"/>
+      <c r="N107" s="12" t="n"/>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P107" s="4" t="inlineStr">
+        <is>
+          <t>content/paths/system-design.yaml: 9 modules, 23 topics, 59 items (9 optional, 16 exercises), about 2 months at an hour a day. Passes the importer's parser; links returned 200 on 2026-10-28 except 3 Cloudflare Learning pages (bot check) and the Instagram sharding post (timed out), still to check by hand. Next: import on production, check in Admin › Catalog, publish.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): mark what's done, add the import features and Data Scientist path
Done: SL-076 backups, SL-083–088 platform admin, SL-095/105/106 official
paths (imported and published). In progress: SL-082 rebrand (awaiting
release), SL-107 Data Scientist path (in OneDrive, not imported yet). New and
done: SL-108 admin import, SL-109 My paths import, SL-110 Markdown in notes.
SL-026 and SL-079 note the Better Stack plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P107" headerRowCount="1">
-  <autoFilter ref="A1:P107"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A1:P111" headerRowCount="1">
+  <autoFilter ref="A1:P111"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Title"/>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P107"/>
+  <dimension ref="A1:P111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3100,7 +3100,11 @@
           <t>README roadmap</t>
         </is>
       </c>
-      <c r="P27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>Chosen: Better Stack free plan (100,000 errors a month, 90 days, works with the Sentry SDKs). Waiting for the two DSNs (gradiaqo-api, gradiaqo-web) from Errors › Applications › Ingest.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -6316,7 +6320,7 @@
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
@@ -6326,7 +6330,9 @@
       </c>
       <c r="L77" s="4" t="n"/>
       <c r="M77" s="12" t="n"/>
-      <c r="N77" s="12" t="n"/>
+      <c r="N77" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O77" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6334,7 +6340,7 @@
       </c>
       <c r="P77" s="4" t="inlineStr">
         <is>
-          <t>The database volume is set to Retain, but that is not a backup. Decide the storage first.</t>
+          <t>CronJob db-backup at 02:00 India time: pg_dump, encrypted with rclone crypt, to OneDrive gradiaqo-backups/, 30 days kept. First backup restored fine.</t>
         </is>
       </c>
     </row>
@@ -6533,7 +6539,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="P80" s="4" t="n"/>
+      <c r="P80" s="4" t="inlineStr">
+        <is>
+          <t>Better Stack free plan: a monitor on https://gradiaqo.com/health with email alerts, in the same account as error tracking (SL-026).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -6712,7 +6722,7 @@
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K83" s="4" t="n"/>
@@ -6724,7 +6734,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="P83" s="4" t="n"/>
+      <c r="P83" s="4" t="inlineStr">
+        <is>
+          <t>Committed on feat/rebrand-gradiaqo (2026-10-28): every visible StudyLog is now Gradiaqo, with the new logo and favicon. To do: merge, build, restart api and web. Internal names (@studylog packages, namespace, database, images) stay.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -6773,13 +6787,15 @@
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K84" s="4" t="n"/>
       <c r="L84" s="4" t="n"/>
       <c r="M84" s="12" t="n"/>
-      <c r="N84" s="12" t="n"/>
+      <c r="N84" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O84" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6838,13 +6854,15 @@
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K85" s="4" t="n"/>
       <c r="L85" s="4" t="n"/>
       <c r="M85" s="12" t="n"/>
-      <c r="N85" s="12" t="n"/>
+      <c r="N85" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O85" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6899,7 +6917,7 @@
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
@@ -6909,7 +6927,9 @@
       </c>
       <c r="L86" s="4" t="n"/>
       <c r="M86" s="12" t="n"/>
-      <c r="N86" s="12" t="n"/>
+      <c r="N86" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O86" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6964,13 +6984,15 @@
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K87" s="4" t="n"/>
       <c r="L87" s="4" t="n"/>
       <c r="M87" s="12" t="n"/>
-      <c r="N87" s="12" t="n"/>
+      <c r="N87" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O87" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7025,13 +7047,15 @@
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K88" s="4" t="n"/>
       <c r="L88" s="4" t="n"/>
       <c r="M88" s="12" t="n"/>
-      <c r="N88" s="12" t="n"/>
+      <c r="N88" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O88" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7086,13 +7110,15 @@
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K89" s="4" t="n"/>
       <c r="L89" s="4" t="n"/>
       <c r="M89" s="12" t="n"/>
-      <c r="N89" s="12" t="n"/>
+      <c r="N89" s="12" t="n">
+        <v>46321</v>
+      </c>
       <c r="O89" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7557,13 +7583,15 @@
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K96" s="4" t="n"/>
       <c r="L96" s="4" t="n"/>
       <c r="M96" s="12" t="n"/>
-      <c r="N96" s="12" t="n"/>
+      <c r="N96" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O96" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7571,7 +7599,7 @@
       </c>
       <c r="P96" s="4" t="inlineStr">
         <is>
-          <t>On 2026-10-24 production had 0 learning paths: a new user finds nothing to study. Do this before any outreach.</t>
+          <t>DSA, AI Engineer and System Design imported and published on production with Admin › Catalog › Import file. Data Scientist is SL-107.</t>
         </is>
       </c>
     </row>
@@ -8207,7 +8235,7 @@
       </c>
       <c r="J106" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K106" s="4" t="inlineStr">
@@ -8217,7 +8245,9 @@
       </c>
       <c r="L106" s="4" t="n"/>
       <c r="M106" s="12" t="n"/>
-      <c r="N106" s="12" t="n"/>
+      <c r="N106" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O106" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -8225,7 +8255,7 @@
       </c>
       <c r="P106" s="4" t="inlineStr">
         <is>
-          <t>content/paths/ai-engineer.yaml: 10 modules, 23 topics, 65 items (15 optional, 12 exercises), about 2–3 months at an hour a day. Passes the importer's parser; all non-YouTube links returned 200 on 2026-10-28, the 5 YouTube links still to check by hand. Next: import on production, check in Admin › Catalog, publish.</t>
+          <t>OneDrive gradiaqo-paths/official/ai-engineer.yaml: imported and published on production.</t>
         </is>
       </c>
     </row>
@@ -8276,7 +8306,7 @@
       </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K107" s="4" t="inlineStr">
@@ -8286,7 +8316,9 @@
       </c>
       <c r="L107" s="4" t="n"/>
       <c r="M107" s="12" t="n"/>
-      <c r="N107" s="12" t="n"/>
+      <c r="N107" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O107" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -8294,7 +8326,281 @@
       </c>
       <c r="P107" s="4" t="inlineStr">
         <is>
-          <t>content/paths/system-design.yaml: 9 modules, 23 topics, 59 items (9 optional, 16 exercises), about 2 months at an hour a day. Passes the importer's parser; links returned 200 on 2026-10-28 except 3 Cloudflare Learning pages (bot check) and the Instagram sharding post (timed out), still to check by hand. Next: import on production, check in Admin › Catalog, publish.</t>
+          <t>OneDrive gradiaqo-paths/official/system-design.yaml: imported and published on production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>SL-107</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Data Scientist learning path</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>An official path: Python and SQL for analysis, statistics, visualisation, machine learning, A/B testing and putting models to work, with 16 LeetCode SQL problems</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="F108" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E108,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K108" s="4" t="inlineStr">
+        <is>
+          <t>SL-095</t>
+        </is>
+      </c>
+      <c r="L108" s="4" t="n"/>
+      <c r="M108" s="12" t="n"/>
+      <c r="N108" s="12" t="n"/>
+      <c r="O108" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P108" s="4" t="inlineStr">
+        <is>
+          <t>Written: OneDrive gradiaqo-paths/official/data-scientist.yaml (path files are not kept in the repo). 9 modules, 62 items, about 160 hours. Next: import with Admin › Catalog › Import file, then publish. Check the OpenIntro link (406 to scripts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>SL-108</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Admin: import a path from a file</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Admin › Catalog › Import file: choose a path YAML file, see what it changes (dry run), import; audit-logged. Replaces running catalog:import with kubectl</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="F109" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E109,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K109" s="4" t="n"/>
+      <c r="L109" s="4" t="n"/>
+      <c r="M109" s="12" t="n"/>
+      <c r="N109" s="12" t="n">
+        <v>46323</v>
+      </c>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P109" s="4" t="inlineStr">
+        <is>
+          <t>POST /admin/catalog/import. Also fixed: re-importing rewrote items whose jsonb details came back with keys in another order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>SL-109</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>My paths: import a path from a file</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>My paths › Import file: anyone imports a path YAML file into their workspace (private, enrolled) or an organization they run, with that catalog's own items</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F110" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E110,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K110" s="4" t="inlineStr">
+        <is>
+          <t>SL-108</t>
+        </is>
+      </c>
+      <c r="L110" s="4" t="n"/>
+      <c r="M110" s="12" t="n"/>
+      <c r="N110" s="12" t="n">
+        <v>46323</v>
+      </c>
+      <c r="O110" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P110" s="4" t="inlineStr">
+        <is>
+          <t>POST /organizations/:organizationId/catalog/import, rate-limited to 60 an hour. Used to import the personal 6-month AI Engineer roadmap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>SL-110</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Notes and instructions show as Markdown</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>The path page showed notes, exercise instructions and answers as raw text, so **bold** and [links](…) appeared with their symbols</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F111" s="4">
+        <f>IFERROR(INDEX(Roadmap!$B$5:$B$16,MATCH(E111,Roadmap!$A$5:$A$16,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K111" s="4" t="n"/>
+      <c r="L111" s="4" t="n"/>
+      <c r="M111" s="12" t="n"/>
+      <c r="N111" s="12" t="n">
+        <v>46323</v>
+      </c>
+      <c r="O111" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="P111" s="4" t="inlineStr">
+        <is>
+          <t>react-markdown + remark-gfm + remark-breaks; HTML never rendered, unsafe links dropped, links open in a new tab.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): SL-082 rebrand, SL-089 SEO basics and SL-107 Data Scientist path done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap.xlsx
+++ b/roadmap.xlsx
@@ -6722,13 +6722,15 @@
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K83" s="4" t="n"/>
       <c r="L83" s="4" t="n"/>
       <c r="M83" s="12" t="n"/>
-      <c r="N83" s="12" t="n"/>
+      <c r="N83" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O83" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -6736,7 +6738,7 @@
       </c>
       <c r="P83" s="4" t="inlineStr">
         <is>
-          <t>Committed on feat/rebrand-gradiaqo (2026-10-28): every visible StudyLog is now Gradiaqo, with the new logo and favicon. To do: merge, build, restart api and web. Internal names (@studylog packages, namespace, database, images) stay.</t>
+          <t>Live on gradiaqo.com: every visible StudyLog is now Gradiaqo, with the new logo and favicon. Internal names (@studylog packages, studylog namespace, database, images, studylog-theme key) stay.</t>
         </is>
       </c>
     </row>
@@ -7173,7 +7175,7 @@
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
@@ -7183,7 +7185,9 @@
       </c>
       <c r="L90" s="4" t="n"/>
       <c r="M90" s="12" t="n"/>
-      <c r="N90" s="12" t="n"/>
+      <c r="N90" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O90" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -7191,7 +7195,7 @@
       </c>
       <c r="P90" s="4" t="inlineStr">
         <is>
-          <t>Today every page is titled "StudyLog", there are no preview tags, and robots.txt and sitemap.xml return the API's 404.</t>
+          <t>robots.txt and sitemap.xml built for the site address, a title and canonical link per public page, Open Graph and Twitter tags with a 1200×630 share card, and an Apple touch icon. Next: submit the sitemap in Search Console (SL-091).</t>
         </is>
       </c>
     </row>
@@ -8377,7 +8381,7 @@
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K108" s="4" t="inlineStr">
@@ -8387,7 +8391,9 @@
       </c>
       <c r="L108" s="4" t="n"/>
       <c r="M108" s="12" t="n"/>
-      <c r="N108" s="12" t="n"/>
+      <c r="N108" s="12" t="n">
+        <v>46323</v>
+      </c>
       <c r="O108" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
@@ -8395,7 +8401,7 @@
       </c>
       <c r="P108" s="4" t="inlineStr">
         <is>
-          <t>Written: OneDrive gradiaqo-paths/official/data-scientist.yaml (path files are not kept in the repo). 9 modules, 62 items, about 160 hours. Next: import with Admin › Catalog › Import file, then publish. Check the OpenIntro link (406 to scripts).</t>
+          <t>OneDrive gradiaqo-paths/official/data-scientist.yaml: imported and published on production.</t>
         </is>
       </c>
     </row>

</xml_diff>